<commit_message>
Migliora foglio Investimenti con 8 righe di esempio
MODIFICHE FOGLIO INVESTIMENTI:
- Aggiunte 8 righe di esempio (invece di solo 3)
- 3 Azioni: Apple, ENI, UniCredit
- 3 ETF: VOO, IWDA, VWCE
- 2 Bond: BTP Italia 2030, BTP 2.5% 2033
- Formule automatiche applicate a tutte le righe
- Colorazione automatica per ogni tipo

CHIARIMENTI DOCUMENTAZIONE:
- Enfatizzato che si possono aggiungere QUANTE RIGHE VUOI
- Chiarito che ogni asset va in una riga separata
- Spiegato come filtrare per tipo
- Suggerito di copiare righe esistenti per mantenere i colori

Risolve: confusione su possibilità di avere più asset per tipo
</commit_message>
<xml_diff>
--- a/Portfolio_Tracker.xlsx
+++ b/Portfolio_Tracker.xlsx
@@ -920,7 +920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1017,6 +1017,18 @@
           <t>Azione</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2">
         <f>IF(A2="Bond","",IFERROR(GOOGLEFINANCE(B2,"price"),""))</f>
         <v/>
@@ -1037,20 +1049,315 @@
         <f>IF(G2&lt;&gt;0,I2/G2*100,"")</f>
         <v/>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>Azione</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BIT:ENI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Eni S.p.A.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3">
+        <f>IF(A3="Bond","",IFERROR(GOOGLEFINANCE(B3,"price"),""))</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>IF(D3&lt;&gt;"",D3*E3,"")</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>IF(AND(D3&lt;&gt;"",F3&lt;&gt;""),D3*F3,"")</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>IF(H3&lt;&gt;"",H3-G3,"")</f>
+        <v/>
+      </c>
+      <c r="J3">
+        <f>IF(G3&lt;&gt;0,I3/G3*100,"")</f>
+        <v/>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Azione</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BIT:UCG</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UniCredit</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4">
+        <f>IF(A4="Bond","",IFERROR(GOOGLEFINANCE(B4,"price"),""))</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>IF(D4&lt;&gt;"",D4*E4,"")</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>IF(AND(D4&lt;&gt;"",F4&lt;&gt;""),D4*F4,"")</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>IF(H4&lt;&gt;"",H4-G4,"")</f>
+        <v/>
+      </c>
+      <c r="J4">
+        <f>IF(G4&lt;&gt;0,I4/G4*100,"")</f>
+        <v/>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Vanguard S&amp;P 500 ETF</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5">
+        <f>IF(A5="Bond","",IFERROR(GOOGLEFINANCE(B5,"price"),""))</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>IF(D5&lt;&gt;"",D5*E5,"")</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>IF(AND(D5&lt;&gt;"",F5&lt;&gt;""),D5*F5,"")</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>IF(H5&lt;&gt;"",H5-G5,"")</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>IF(G5&lt;&gt;0,I5/G5*100,"")</f>
+        <v/>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>ETF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EPA:IWDA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>iShares Core MSCI World</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6">
+        <f>IF(A6="Bond","",IFERROR(GOOGLEFINANCE(B6,"price"),""))</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>IF(D6&lt;&gt;"",D6*E6,"")</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>IF(AND(D6&lt;&gt;"",F6&lt;&gt;""),D6*F6,"")</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>IF(H6&lt;&gt;"",H6-G6,"")</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>IF(G6&lt;&gt;0,I6/G6*100,"")</f>
+        <v/>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>ETF</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AMS:VWCE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE All-World</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7">
+        <f>IF(A7="Bond","",IFERROR(GOOGLEFINANCE(B7,"price"),""))</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>IF(D7&lt;&gt;"",D7*E7,"")</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>IF(AND(D7&lt;&gt;"",F7&lt;&gt;""),D7*F7,"")</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>IF(H7&lt;&gt;"",H7-G7,"")</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>IF(G7&lt;&gt;0,I7/G7*100,"")</f>
+        <v/>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Bond</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IT0005423745</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BTP Italia 2030</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8">
+        <f>IF(A8="Bond","",IFERROR(GOOGLEFINANCE(B8,"price"),""))</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IF(D8&lt;&gt;"",D8*E8,"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IF(AND(D8&lt;&gt;"",F8&lt;&gt;""),D8*F8,"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IF(H8&lt;&gt;"",H8-G8,"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IF(G8&lt;&gt;0,I8/G8*100,"")</f>
+        <v/>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>31/12/2030</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>Bond</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BTP 2.5% 2033</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9">
+        <f>IF(A9="Bond","",IFERROR(GOOGLEFINANCE(B9,"price"),""))</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>IF(D9&lt;&gt;"",D9*E9,"")</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>IF(AND(D9&lt;&gt;"",F9&lt;&gt;""),D9*F9,"")</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>IF(H9&lt;&gt;"",H9-G9,"")</f>
+        <v/>
+      </c>
+      <c r="J9">
+        <f>IF(G9&lt;&gt;0,I9/G9*100,"")</f>
+        <v/>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>01/12/2033</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>